<commit_message>
Modified preprocessing and dataset validation to match the new data structure; created two new folders in preprocessed data
</commit_message>
<xml_diff>
--- a/Data/raw/TST_Mannino_2023-10_QS/TST_2023-10_QS_metadata.xlsx
+++ b/Data/raw/TST_Mannino_2023-10_QS/TST_2023-10_QS_metadata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oros\Desktop\dataset_upload\TST_Mannino_2023-10_QS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4850C9CB-A961-45DC-8E24-B61496B13C87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5598DDD8-D9FB-4F83-A960-B4317CC92EDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="15" windowWidth="20640" windowHeight="11040" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -893,6 +893,9 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -915,9 +918,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -925,21 +925,7 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="6">
     <dxf>
       <fill>
         <patternFill>
@@ -1513,55 +1499,55 @@
     <row r="1" spans="1:41" s="2" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="11"/>
       <c r="B1" s="11"/>
-      <c r="C1" s="26" t="s">
+      <c r="C1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="26"/>
-      <c r="M1" s="26"/>
-      <c r="N1" s="26"/>
-      <c r="O1" s="26"/>
-      <c r="P1" s="26"/>
-      <c r="Q1" s="26"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
       <c r="R1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="S1" s="27" t="s">
+      <c r="S1" s="28" t="s">
         <v>144</v>
       </c>
-      <c r="T1" s="27"/>
-      <c r="U1" s="27"/>
-      <c r="V1" s="27"/>
-      <c r="W1" s="27"/>
-      <c r="X1" s="27"/>
-      <c r="Y1" s="27"/>
-      <c r="Z1" s="27"/>
-      <c r="AA1" s="27"/>
-      <c r="AB1" s="27"/>
-      <c r="AC1" s="27"/>
-      <c r="AD1" s="27"/>
-      <c r="AE1" s="27"/>
-      <c r="AF1" s="27"/>
-      <c r="AG1" s="27"/>
-      <c r="AH1" s="27"/>
-      <c r="AI1" s="27"/>
-      <c r="AJ1" s="27"/>
-      <c r="AK1" s="27"/>
-      <c r="AL1" s="25" t="s">
+      <c r="T1" s="28"/>
+      <c r="U1" s="28"/>
+      <c r="V1" s="28"/>
+      <c r="W1" s="28"/>
+      <c r="X1" s="28"/>
+      <c r="Y1" s="28"/>
+      <c r="Z1" s="28"/>
+      <c r="AA1" s="28"/>
+      <c r="AB1" s="28"/>
+      <c r="AC1" s="28"/>
+      <c r="AD1" s="28"/>
+      <c r="AE1" s="28"/>
+      <c r="AF1" s="28"/>
+      <c r="AG1" s="28"/>
+      <c r="AH1" s="28"/>
+      <c r="AI1" s="28"/>
+      <c r="AJ1" s="28"/>
+      <c r="AK1" s="28"/>
+      <c r="AL1" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="AM1" s="25"/>
-      <c r="AN1" s="22" t="s">
+      <c r="AM1" s="26"/>
+      <c r="AN1" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="AO1" s="23"/>
+      <c r="AO1" s="24"/>
     </row>
     <row r="2" spans="1:41" s="2" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="21" t="s">
@@ -1720,7 +1706,7 @@
       <c r="O3" s="13"/>
       <c r="P3" s="13"/>
       <c r="Q3" s="13"/>
-      <c r="R3" s="30" t="s">
+      <c r="R3" s="22" t="s">
         <v>156</v>
       </c>
       <c r="S3" s="12" t="s">
@@ -2101,14 +2087,14 @@
       <c r="S7" s="1"/>
     </row>
     <row r="8" spans="1:41" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="24" t="s">
+      <c r="A8" s="25" t="s">
         <v>148</v>
       </c>
-      <c r="B8" s="24"/>
+      <c r="B8" s="25"/>
     </row>
     <row r="9" spans="1:41" x14ac:dyDescent="0.3">
-      <c r="A9" s="24"/>
-      <c r="B9" s="24"/>
+      <c r="A9" s="25"/>
+      <c r="B9" s="25"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
@@ -2120,32 +2106,32 @@
     <mergeCell ref="S1:AK1"/>
   </mergeCells>
   <conditionalFormatting sqref="G3">
-    <cfRule type="expression" dxfId="7" priority="6">
+    <cfRule type="expression" dxfId="5" priority="6">
       <formula>F3="QS"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3 O3 AN3:AO3">
-    <cfRule type="expression" dxfId="6" priority="9">
+    <cfRule type="expression" dxfId="4" priority="9">
       <formula>$F$3="FA"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I3">
-    <cfRule type="expression" dxfId="5" priority="5">
+    <cfRule type="expression" dxfId="3" priority="5">
       <formula>F3="OT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J3 P3">
-    <cfRule type="expression" dxfId="4" priority="3">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>I3="Other"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K3">
-    <cfRule type="expression" dxfId="3" priority="7">
+    <cfRule type="expression" dxfId="1" priority="7">
       <formula>OR(G3="fracture", H3="fracture")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U3">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>S3="Other polymers"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2228,29 +2214,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="27" t="s">
         <v>101</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="29" t="s">
+      <c r="B1" s="27"/>
+      <c r="C1" s="30" t="s">
         <v>61</v>
       </c>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="27" t="s">
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="28" t="s">
         <v>102</v>
       </c>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="25" t="s">
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="26" t="s">
         <v>103</v>
       </c>
-      <c r="K1" s="25"/>
-      <c r="L1" s="28" t="s">
+      <c r="K1" s="26"/>
+      <c r="L1" s="29" t="s">
         <v>104</v>
       </c>
-      <c r="M1" s="28"/>
+      <c r="M1" s="29"/>
     </row>
     <row r="2" spans="1:13" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
@@ -2305,10 +2291,10 @@
       <c r="E3" s="13"/>
       <c r="F3" s="13"/>
       <c r="G3" s="12">
+        <v>13.11</v>
+      </c>
+      <c r="H3" s="12">
         <v>3.18</v>
-      </c>
-      <c r="H3" s="12">
-        <v>13.11</v>
       </c>
       <c r="I3" s="13"/>
       <c r="J3" s="19"/>
@@ -2328,10 +2314,10 @@
       <c r="E4" s="13"/>
       <c r="F4" s="13"/>
       <c r="G4" s="12">
+        <v>12.95</v>
+      </c>
+      <c r="H4" s="12">
         <v>3.24</v>
-      </c>
-      <c r="H4" s="12">
-        <v>12.95</v>
       </c>
       <c r="I4" s="13"/>
       <c r="J4" s="19"/>
@@ -2351,10 +2337,10 @@
       <c r="E5" s="13"/>
       <c r="F5" s="13"/>
       <c r="G5" s="12">
+        <v>12.93</v>
+      </c>
+      <c r="H5" s="12">
         <v>3.24</v>
-      </c>
-      <c r="H5" s="12">
-        <v>12.93</v>
       </c>
       <c r="I5" s="13"/>
       <c r="J5" s="19"/>
@@ -2374,10 +2360,10 @@
       <c r="E6" s="13"/>
       <c r="F6" s="13"/>
       <c r="G6" s="12">
+        <v>12.95</v>
+      </c>
+      <c r="H6" s="12">
         <v>3.4</v>
-      </c>
-      <c r="H6" s="12">
-        <v>12.95</v>
       </c>
       <c r="I6" s="13"/>
       <c r="J6" s="19"/>

</xml_diff>